<commit_message>
18 MAY add note
</commit_message>
<xml_diff>
--- a/BFC_lithic_data.xlsx
+++ b/BFC_lithic_data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuanx\Desktop\Bianfu_Cave_lithic_analysis\BFC_lithic_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A03D34-61DB-4FFB-AFDB-282D41718D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF65425-2169-41FA-8AB5-D7208EA0DB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{13ADFA50-5ED3-4C75-A674-4AB884131A0C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{13ADFA50-5ED3-4C75-A674-4AB884131A0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Core" sheetId="1" r:id="rId1"/>
     <sheet name="Flake" sheetId="3" r:id="rId2"/>
     <sheet name="Tool" sheetId="4" r:id="rId3"/>
     <sheet name="Chunk" sheetId="2" r:id="rId4"/>
+    <sheet name="Note" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Chunk!$A$1:$K$925</definedName>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10668" uniqueCount="1577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10669" uniqueCount="1578">
   <si>
     <t>No.</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -4937,6 +4938,11 @@
   </si>
   <si>
     <t>12</t>
+  </si>
+  <si>
+    <t>During excavation, all specimens that could be recorded with three-dimensional coordinates were numbered. 
+Specimens without coordinates, which were usually heavily cemented, were numbered subsequently during laboratory work. Consequently, the order of specimen numbers does not fully correspond to the stratigraphic sequence of excavation layers.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -5088,7 +5094,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5157,6 +5163,9 @@
     </xf>
     <xf numFmtId="179" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -68572,4 +68581,23 @@
     <ignoredError sqref="B2:B925" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{679792E4-5CBB-4A0A-90EC-1190B3066A67}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="49.125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="102.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>